<commit_message>
fix: bulk order generation process and UI improvements
</commit_message>
<xml_diff>
--- a/apps/frontend/public/bulk_order_template.xlsx
+++ b/apps/frontend/public/bulk_order_template.xlsx
@@ -400,171 +400,223 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:O4"/>
   <cols>
-    <col min="1" max="1" width="22.83203125" customWidth="1"/>
-    <col min="2" max="2" width="16.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="18.83203125" customWidth="1"/>
-    <col min="5" max="5" width="28.83203125" customWidth="1"/>
-    <col min="6" max="6" width="22.83203125" customWidth="1"/>
-    <col min="7" max="7" width="10.83203125" customWidth="1"/>
-    <col min="8" max="8" width="14.83203125" customWidth="1"/>
-    <col min="9" max="9" width="10.83203125" customWidth="1"/>
-    <col min="10" max="10" width="12.83203125" customWidth="1"/>
-    <col min="11" max="11" width="24.83203125" customWidth="1"/>
+    <col min="1" max="1" width="14.83203125" customWidth="1"/>
+    <col min="2" max="2" width="22.83203125" customWidth="1"/>
+    <col min="3" max="3" width="16.83203125" customWidth="1"/>
+    <col min="4" max="4" width="16.83203125" customWidth="1"/>
+    <col min="5" max="5" width="16.83203125" customWidth="1"/>
+    <col min="6" max="6" width="16.83203125" customWidth="1"/>
+    <col min="7" max="7" width="32.83203125" customWidth="1"/>
+    <col min="8" max="8" width="28.83203125" customWidth="1"/>
+    <col min="9" max="9" width="22.83203125" customWidth="1"/>
+    <col min="10" max="10" width="8.83203125" customWidth="1"/>
+    <col min="11" max="11" width="12.83203125" customWidth="1"/>
+    <col min="12" max="12" width="10.83203125" customWidth="1"/>
+    <col min="13" max="13" width="12.83203125" customWidth="1"/>
+    <col min="14" max="14" width="12.83203125" customWidth="1"/>
+    <col min="15" max="15" width="24.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
+        <v>Order Code</v>
+      </c>
+      <c r="B1" t="str">
         <v>Customer Name</v>
       </c>
-      <c r="B1" t="str">
+      <c r="C1" t="str">
         <v>Phone</v>
       </c>
-      <c r="C1" t="str">
+      <c r="D1" t="str">
         <v>City</v>
       </c>
-      <c r="D1" t="str">
+      <c r="E1" t="str">
+        <v>Area</v>
+      </c>
+      <c r="F1" t="str">
         <v>Governorate</v>
       </c>
-      <c r="E1" t="str">
+      <c r="G1" t="str">
+        <v>Address</v>
+      </c>
+      <c r="H1" t="str">
         <v>Product Name</v>
       </c>
-      <c r="F1" t="str">
+      <c r="I1" t="str">
         <v>SKU</v>
       </c>
-      <c r="G1" t="str">
+      <c r="J1" t="str">
         <v>Size</v>
       </c>
-      <c r="H1" t="str">
+      <c r="K1" t="str">
         <v>Color</v>
       </c>
-      <c r="I1" t="str">
+      <c r="L1" t="str">
         <v>Quantity</v>
       </c>
-      <c r="J1" t="str">
+      <c r="M1" t="str">
         <v>Price</v>
       </c>
-      <c r="K1" t="str">
+      <c r="N1" t="str">
+        <v>COD</v>
+      </c>
+      <c r="O1" t="str">
         <v>Notes</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
+        <v>38124947</v>
+      </c>
+      <c r="B2" t="str">
         <v>Ahmed Mohamed</v>
       </c>
-      <c r="B2" t="str">
+      <c r="C2" t="str">
         <v>01001234567</v>
       </c>
-      <c r="C2" t="str">
+      <c r="D2" t="str">
         <v>Nasr City</v>
       </c>
-      <c r="D2" t="str">
+      <c r="E2" t="str">
+        <v>الحي السابع</v>
+      </c>
+      <c r="F2" t="str">
         <v>Cairo</v>
       </c>
-      <c r="E2" t="str">
+      <c r="G2" t="str">
+        <v>العبور فيلا 38</v>
+      </c>
+      <c r="H2" t="str">
         <v>Nike Air Max 270</v>
       </c>
-      <c r="F2" t="str">
+      <c r="I2" t="str">
         <v>NIKE-AM270-BLK</v>
       </c>
-      <c r="G2" t="str">
+      <c r="J2" t="str">
         <v>42</v>
       </c>
-      <c r="H2" t="str">
+      <c r="K2" t="str">
         <v>Black</v>
       </c>
-      <c r="I2" s="1">
+      <c r="L2" s="1">
         <v>2</v>
       </c>
-      <c r="J2" s="2">
+      <c r="M2" s="2">
         <v>150</v>
       </c>
-      <c r="K2" t="str">
+      <c r="N2" s="2">
+        <v>300</v>
+      </c>
+      <c r="O2" t="str">
         <v>توصيل سريع</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
+        <v>38124946</v>
+      </c>
+      <c r="B3" t="str">
         <v>Sara Ali</v>
       </c>
-      <c r="B3" t="str">
+      <c r="C3" t="str">
         <v>01112223333</v>
       </c>
-      <c r="C3" t="str">
+      <c r="D3" t="str">
         <v>Mohandessin</v>
       </c>
-      <c r="D3" t="str">
+      <c r="E3" t="str">
+        <v/>
+      </c>
+      <c r="F3" t="str">
         <v>Giza</v>
       </c>
-      <c r="E3" t="str">
+      <c r="G3" t="str">
+        <v>٣شارع عبد الحميد</v>
+      </c>
+      <c r="H3" t="str">
         <v>Adidas Ultraboost</v>
       </c>
-      <c r="F3" t="str">
+      <c r="I3" t="str">
         <v>AD-UBS-WHT</v>
       </c>
-      <c r="G3" t="str">
+      <c r="J3" t="str">
         <v>38</v>
       </c>
-      <c r="H3" t="str">
+      <c r="K3" t="str">
         <v>White</v>
       </c>
-      <c r="I3" s="1">
+      <c r="L3" s="1">
         <v>1</v>
       </c>
-      <c r="J3" s="2">
+      <c r="M3" s="2">
         <v>200</v>
       </c>
-      <c r="K3" t="str">
+      <c r="N3" s="2">
+        <v>200</v>
+      </c>
+      <c r="O3" t="str">
         <v/>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
+        <v>38124943</v>
+      </c>
+      <c r="B4" t="str">
         <v>Mohamed Khaled</v>
       </c>
-      <c r="B4" t="str">
+      <c r="C4" t="str">
         <v>01009998877</v>
       </c>
-      <c r="C4" t="str">
+      <c r="D4" t="str">
         <v>Maadi</v>
       </c>
-      <c r="D4" t="str">
+      <c r="E4" t="str">
+        <v>بئر ام سلطان</v>
+      </c>
+      <c r="F4" t="str">
         <v>Cairo</v>
       </c>
-      <c r="E4" t="str">
+      <c r="G4" t="str">
+        <v>46 ش كامل همام</v>
+      </c>
+      <c r="H4" t="str">
         <v>Puma T-Shirt</v>
       </c>
-      <c r="F4" t="str">
+      <c r="I4" t="str">
         <v>PU-TS-RED</v>
       </c>
-      <c r="G4" t="str">
+      <c r="J4" t="str">
         <v>L</v>
       </c>
-      <c r="H4" t="str">
+      <c r="K4" t="str">
         <v>Red</v>
       </c>
-      <c r="I4" s="1">
+      <c r="L4" s="1">
         <v>3</v>
       </c>
-      <c r="J4" s="2">
+      <c r="M4" s="2">
         <v>75.5</v>
       </c>
-      <c r="K4" t="str">
+      <c r="N4" s="2">
+        <v>226.5</v>
+      </c>
+      <c r="O4" t="str">
         <v>مقاس كبير</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O4"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A36"/>
+  <dimension ref="A1:A38"/>
   <cols>
     <col min="1" max="1" width="80.83203125" customWidth="1"/>
   </cols>
@@ -601,77 +653,77 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>4. Quantity and Price MUST be numbers only. Do not add currency symbols.</v>
+        <v>4. Columns: Customer Name, Phone, City, Area, Governorate, Address, Product Name, SKU, Size, Color, Quantity, Price, COD, Notes.</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>5. Notes column is optional - you can leave it empty.</v>
+        <v>5. Quantity, Price, and COD MUST be numbers only. Do not add currency symbols.</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>6. Save the file and upload it from the Bulk Orders page.</v>
+        <v>6. Area, Address, and Notes columns are optional.</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>7. Supported formats: .xlsx, .xls, .csv</v>
+        <v>7. Save the file and upload it from the Bulk Orders page.</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v/>
+        <v>8. Supports both English and Arabic column headers (.xlsx, .xls, .csv).</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>عربي:</v>
+        <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>-١ .املأ بيانات الطلبات في ورقة "Orders" بدءاً من الصف ٢ (أسفل العنوان)</v>
+        <v>عربي:</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>-٢ .احذف صفوف بيانات العينة (الصفوف ٢-٤) قبل إضافة بياناتك</v>
+        <v>-١ .املأ بيانات الطلبات في ورقة "Orders" بدءاً من الصف ٢ (أسفل العنوان)</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>-٣ .لا تقم بتعديل أو حذف صف العنوان (الصف ١)</v>
+        <v>-٢ .احذف صفوف بيانات العينة (الصفوف ٢-٤) قبل إضافة بياناتك</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>-٤ .الكمية والسعر يجب أن يكونا أرقاماً فقط. لا تضف رموز العملة</v>
+        <v>-٣ .لا تقم بتعديل أو حذف صف العنوان (الصف ١)</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>-٥ .عمود الملاحظات اختياري - يمكنك تركه فارغاً</v>
+        <v>-٤ .الأعمدة: اسم العميل، الهاتف، المدينة، المنطقة، المحافظة، العنوان، اسم المنتج، SKU، المقاس، اللون، الكمية، السعر، المبلغ، ملاحظات</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>-٦ .احفظ الملف وارفعه من صفحة الطلبات المجمعة</v>
+        <v>-٥ .الكمية والسعر والمبلغ يجب أن يكونا أرقاماً فقط. لا تضف رموز العملة</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>-٧ .الصيغ المدعومة: xlsx. , xls. , csv.</v>
+        <v>-٦ .حقول المنطقة والعنوان والملاحظات اختيارية</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v/>
+        <v>-٧ .احفظ الملف وارفعه من صفحة الطلبات المجمعة</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>COLUMN NAMES (English / Arabic) / أسماء الأعمدة (إنجليزي / عربي):</v>
+        <v>-٨ .يدعم العناوين بالإنجليزية والعربية (xlsx. , xls. , csv.)</v>
       </c>
     </row>
     <row r="22">
@@ -681,77 +733,87 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Customer Name    =    اسم العميل</v>
+        <v>COLUMN MAPPING / خريطة الأعمدة (النظام يتعرف على كلا الإسمين):</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Phone            =    الهاتف</v>
+        <v/>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>City             =    المدينة</v>
+        <v>Customer Name  =  اسم العميل  /  اسم المستلم</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>Governorate      =    المحافظة</v>
+        <v>Phone          =  الهاتف  /  رقم الهاتف</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>Product Name     =    اسم المنتج</v>
+        <v>City           =  المدينة</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>SKU              =    SKU</v>
+        <v>Area           =  المنطقة</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>Size             =    المقاس</v>
+        <v>Governorate    =  المحافظة</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Color            =    اللون</v>
+        <v>Address        =  العنوان</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Quantity         =    الكمية</v>
+        <v>Product Name   =  اسم المنتج  /  المنتج  /  محتوى الطلب</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Price            =    السعر</v>
+        <v>SKU            =  SKU</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Notes            =    ملاحظات</v>
+        <v>Size           =  المقاس</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v/>
+        <v>Color          =  اللون</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>NOTE: You can use EITHER English OR Arabic column headers in your own files.</v>
+        <v>Quantity       =  الكمية</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>ملاحظة: يمكنك استخدام العناوين بالإنجليزية أو العربية في ملفاتك.</v>
+        <v>Price          =  السعر</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>COD            =  المبلغ المطلوب تحصيله</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>Notes          =  ملاحظات</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A36"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A38"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>